<commit_message>
Nuevo codigo para lectura de imagen sin configuracion complicada tanto local como para citrix
</commit_message>
<xml_diff>
--- a/Pruebas/Archivos/Template/Colombia/Template_HRC_Cruz_Verde.xlsx
+++ b/Pruebas/Archivos/Template/Colombia/Template_HRC_Cruz_Verde.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -479,7 +479,7 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="29" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="G6" s="5" t="n">
-        <v>842873505</v>
+        <v>860873505</v>
       </c>
     </row>
     <row r="7">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="G7" s="5" t="n">
-        <v>842873505</v>
+        <v>860873505</v>
       </c>
     </row>
     <row r="8">
@@ -583,7 +583,7 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10/12/2025</t>
+          <t>22/12/2025</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="F12" s="6" t="n">
-        <v>842873505</v>
+        <v>860873505</v>
       </c>
     </row>
     <row r="13"/>
@@ -1047,11 +1047,11 @@
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>MENORES VALORES</t>
+          <t>PMP1271749</t>
         </is>
       </c>
       <c r="E37" s="6" t="n">
-        <v>788.1800000146031</v>
+        <v>8999999.479999997</v>
       </c>
       <c r="F37" s="10" t="inlineStr">
         <is>
@@ -1060,15 +1060,15 @@
       </c>
       <c r="G37" s="10" t="inlineStr">
         <is>
-          <t>388</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H37" s="6" t="n">
-        <v>788.1800000146031</v>
+        <v>8999999.479999997</v>
       </c>
       <c r="I37" s="11" t="inlineStr">
         <is>
-          <t>MENORES VALORES</t>
+          <t>Saldo FC PMP1271749</t>
         </is>
       </c>
     </row>
@@ -1088,12 +1088,12 @@
       </c>
       <c r="F38" s="10" t="inlineStr">
         <is>
-          <t>Myr Vlr Pagado</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
       <c r="G38" s="10" t="inlineStr">
         <is>
-          <t>388</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H38" s="6" t="n">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Myr Vlr Pagado PMP1271750</t>
+          <t>Saldo FC PMP1271750</t>
         </is>
       </c>
     </row>
@@ -1121,12 +1121,12 @@
       </c>
       <c r="F39" s="10" t="inlineStr">
         <is>
-          <t>Menor Vlr Pagado</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
       <c r="G39" s="10" t="inlineStr">
         <is>
-          <t>CSR</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H39" s="6" t="n">
@@ -1134,7 +1134,337 @@
       </c>
       <c r="I39" s="11" t="inlineStr">
         <is>
-          <t>Menor Vlr Pagado PMP1275487</t>
+          <t>Myr Vlr Pagado PMP1275487</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>PMP1278368</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="n">
+        <v>9000294.819999993</v>
+      </c>
+      <c r="F40" s="10" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+      <c r="G40" s="10" t="inlineStr">
+        <is>
+          <t>987</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="n">
+        <v>9000294.819999993</v>
+      </c>
+      <c r="I40" s="11" t="inlineStr">
+        <is>
+          <t>Saldo FC PMP1278368</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>PMP1275488</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="n">
+        <v>433.6200000047684</v>
+      </c>
+      <c r="F41" s="10" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+      <c r="G41" s="10" t="inlineStr">
+        <is>
+          <t>384</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="n">
+        <v>433.6200000047684</v>
+      </c>
+      <c r="I41" s="11" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>PMP1275489</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="F42" s="10" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+      <c r="G42" s="10" t="inlineStr">
+        <is>
+          <t>384</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="I42" s="11" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>PMP1275491</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="n">
+        <v>234.179999999702</v>
+      </c>
+      <c r="F43" s="10" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+      <c r="G43" s="10" t="inlineStr">
+        <is>
+          <t>384</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="n">
+        <v>234.179999999702</v>
+      </c>
+      <c r="I43" s="11" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="C44" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="inlineStr">
+        <is>
+          <t>PMP1278364</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="n">
+        <v>14.48000000044703</v>
+      </c>
+      <c r="F44" s="10" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+      <c r="G44" s="10" t="inlineStr">
+        <is>
+          <t>384</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="n">
+        <v>14.48000000044703</v>
+      </c>
+      <c r="I44" s="11" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D45" s="10" t="inlineStr">
+        <is>
+          <t>PMP1278365</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="n">
+        <v>148.8000000007451</v>
+      </c>
+      <c r="F45" s="10" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+      <c r="G45" s="10" t="inlineStr">
+        <is>
+          <t>384</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="n">
+        <v>148.8000000007451</v>
+      </c>
+      <c r="I45" s="11" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="C46" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D46" s="10" t="inlineStr">
+        <is>
+          <t>PMP1278366</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="n">
+        <v>104.5200000032783</v>
+      </c>
+      <c r="F46" s="10" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+      <c r="G46" s="10" t="inlineStr">
+        <is>
+          <t>384</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="n">
+        <v>104.5200000032783</v>
+      </c>
+      <c r="I46" s="11" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="C47" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D47" s="10" t="inlineStr">
+        <is>
+          <t>PMP1275485</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="n">
+        <v>-0.199999988079071</v>
+      </c>
+      <c r="F47" s="10" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+      <c r="G47" s="10" t="inlineStr">
+        <is>
+          <t>WOB</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="n">
+        <v>-0.199999988079071</v>
+      </c>
+      <c r="I47" s="11" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="C48" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D48" s="10" t="inlineStr">
+        <is>
+          <t>PMP1275486</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="n">
+        <v>-455.5199999958277</v>
+      </c>
+      <c r="F48" s="10" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+      <c r="G48" s="10" t="inlineStr">
+        <is>
+          <t>WOB</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="n">
+        <v>-455.5199999958277</v>
+      </c>
+      <c r="I48" s="11" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="C49" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D49" s="10" t="inlineStr">
+        <is>
+          <t>PMP1278363</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F49" s="10" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+      <c r="G49" s="10" t="inlineStr">
+        <is>
+          <t>WOB</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I49" s="11" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1511,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>50883742</v>
+        <v>59883742</v>
       </c>
     </row>
     <row r="4">
@@ -1321,7 +1651,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>80917123</v>
+        <v>89917123</v>
       </c>
     </row>
     <row r="18">

</xml_diff>